<commit_message>
Complete monthly report B22-B34 integration
</commit_message>
<xml_diff>
--- a/data sample/DATA SAMPLE THANG/1. BÁO CÁO MBB_HUNG.xlsx
+++ b/data sample/DATA SAMPLE THANG/1. BÁO CÁO MBB_HUNG.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quyng\Documents\TOOL TỔNG HỢP BÁO CÁO\BÁO CÁO TUẦN 29\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quyng\Documents\TOOL TỔNG HỢP BÁO CÁO\VNPT REPORT\data sample\DATA SAMPLE THANG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FA68A25-7E7D-40F6-94DF-FEA1D64B27DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B1B66C-139E-41B3-973F-A47EF56FE42E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kết quả chung" sheetId="8" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="122">
   <si>
     <t>Khu vực</t>
   </si>
@@ -404,6 +404,18 @@
   </si>
   <si>
     <t>KẾT QUẢ CHI TIẾT QoS / QoE</t>
+  </si>
+  <si>
+    <t>B10_HUNG</t>
+  </si>
+  <si>
+    <t>B13_HUNG</t>
+  </si>
+  <si>
+    <t>B14_HUNG</t>
+  </si>
+  <si>
+    <t>B15_HUNG</t>
   </si>
 </sst>
 </file>
@@ -534,7 +546,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="55">
+  <borders count="57">
     <border>
       <left/>
       <right/>
@@ -1218,11 +1230,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF163A5C"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF9EADBA"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1471,12 +1501,245 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="47">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB4C6E7"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1700,6 +1963,217 @@
         <name val="Times New Roman"/>
         <scheme val="none"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFB7C3D0"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFB7C3D0"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF163A5C"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF163A5C"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFB7C3D0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
       <numFmt numFmtId="164" formatCode="00"/>
       <fill>
         <patternFill patternType="solid">
@@ -1813,6 +2287,117 @@
       </border>
     </dxf>
     <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF163A5C"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFB7C3D0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB4C6E7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1824,175 +2409,71 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color rgb="FF222222"/>
+        <color theme="1"/>
         <name val="Times New Roman"/>
+        <family val="1"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="1" formatCode="0"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="0"/>
         </patternFill>
       </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color rgb="FF222222"/>
+        <color theme="1"/>
         <name val="Times New Roman"/>
+        <family val="1"/>
         <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
+    </dxf>
+    <dxf>
+      <border>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -2028,217 +2509,6 @@
         </left>
         <right style="thin">
           <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFB7C3D0"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF222222"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFB7C3D0"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="medium">
-          <color rgb="FF163A5C"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFB7C3D0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color rgb="FF163A5C"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF4472C4"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
         </right>
         <top/>
         <bottom/>
@@ -2628,234 +2898,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="medium">
-          <color rgb="FF163A5C"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFB7C3D0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB4C6E7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB4C6E7"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -2875,20 +2917,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{08017804-8AF8-48ED-9408-1CC56682718D}" name="b1_hung" displayName="b1_hung" ref="A4:D6" totalsRowShown="0" headerRowDxfId="46" dataDxfId="44" headerRowBorderDxfId="45" tableBorderDxfId="43" totalsRowBorderDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{08017804-8AF8-48ED-9408-1CC56682718D}" name="b1_hung" displayName="b1_hung" ref="A4:D6" totalsRowShown="0" headerRowDxfId="35" dataDxfId="33" headerRowBorderDxfId="34" tableBorderDxfId="32" totalsRowBorderDxfId="31">
   <autoFilter ref="A4:D6" xr:uid="{08017804-8AF8-48ED-9408-1CC56682718D}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{82B39A46-8A34-4668-969A-CB1C9A5CDC82}" name="STT" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{3B583058-53A2-4022-83D8-766AA41A2746}" name="Đơn vị" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{4E801DA8-F720-4406-98CA-F5E7A9C551EB}" name="QoS" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{C7638FA1-E728-4FE1-9093-5F43A6514EA9}" name="QoE" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{82B39A46-8A34-4668-969A-CB1C9A5CDC82}" name="STT" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{3B583058-53A2-4022-83D8-766AA41A2746}" name="Đơn vị" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{4E801DA8-F720-4406-98CA-F5E7A9C551EB}" name="QoS" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{C7638FA1-E728-4FE1-9093-5F43A6514EA9}" name="QoE" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BBD08E6D-42DC-46D6-92D9-31C0F836739D}" name="b2_hung" displayName="b2_hung" ref="A3:C7" totalsRowShown="0" headerRowDxfId="37" tableBorderDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BBD08E6D-42DC-46D6-92D9-31C0F836739D}" name="b2_hung" displayName="b2_hung" ref="A3:C7" totalsRowShown="0" headerRowDxfId="26" tableBorderDxfId="25">
   <autoFilter ref="A3:C7" xr:uid="{BBD08E6D-42DC-46D6-92D9-31C0F836739D}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{CCB39EF0-ABD6-4672-AA19-F0146D60E6C2}" name="Tỉnh"/>
@@ -2900,68 +2942,68 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8A05E8FF-0801-48F4-8A03-2065EF193CE7}" name="b3_hung" displayName="b3_hung" ref="A3:H12" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34" tableBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8A05E8FF-0801-48F4-8A03-2065EF193CE7}" name="b3_hung" displayName="b3_hung" ref="A3:H12" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45" tableBorderDxfId="44">
   <autoFilter ref="A3:H12" xr:uid="{8A05E8FF-0801-48F4-8A03-2065EF193CE7}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1DD15225-4E1F-4E43-809E-F6E867610D30}" name="STT" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{F490C3E3-D346-4A06-A474-95147B3E7183}" name="QoS, QoE" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{2F5A7158-E40A-4AEF-BDB7-AAB5EA94A241}" name="Thành phần" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{EC662DDA-7B49-4F8A-A5AB-D3D7DC9D0F3A}" name="Điểm thành phần" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{010D9CD0-4E3D-459B-89BE-3192C944FEC9}" name="Tổng (VB: 22/QĐ-VNPT-TNH)" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{75C4D620-58CB-4A1F-AD46-AF24D5951EE9}" name="Điểm tổng (%)" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{1A771FEE-7377-4D60-B5C3-F00FEA9C1941}" name="Đánh giá" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{00717DD7-2B8E-4212-B758-5E741C46BB14}" name="Xếp hạng" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{1DD15225-4E1F-4E43-809E-F6E867610D30}" name="STT" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{F490C3E3-D346-4A06-A474-95147B3E7183}" name="QoS, QoE" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{2F5A7158-E40A-4AEF-BDB7-AAB5EA94A241}" name="Thành phần" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{EC662DDA-7B49-4F8A-A5AB-D3D7DC9D0F3A}" name="Điểm thành phần" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{010D9CD0-4E3D-459B-89BE-3192C944FEC9}" name="Tổng (VB: 22/QĐ-VNPT-TNH)" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{75C4D620-58CB-4A1F-AD46-AF24D5951EE9}" name="Điểm tổng (%)" dataDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{1A771FEE-7377-4D60-B5C3-F00FEA9C1941}" name="Đánh giá" dataDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{00717DD7-2B8E-4212-B758-5E741C46BB14}" name="Xếp hạng" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{EDBB591E-3AEF-4EEA-AEF8-B76A85739C69}" name="b4_hung" displayName="b4_hung" ref="A4:D10" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{EDBB591E-3AEF-4EEA-AEF8-B76A85739C69}" name="b4_hung" displayName="b4_hung" ref="A4:D10" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="18" tableBorderDxfId="19">
   <autoFilter ref="A4:D10" xr:uid="{EDBB591E-3AEF-4EEA-AEF8-B76A85739C69}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{26FE1E68-CD21-4445-80E0-A77866151FAB}" name="Khu vực" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{6D6F3738-0F8B-45BF-A515-A2A321F895EA}" name="Trạm" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{015C2645-BD78-45F2-98E9-00B03187980C}" name="Nguyên nhân" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{1175C761-AE1A-480A-9F1A-A8F410E010A6}" name="Hiện trạng / Đã xử lý" dataDxfId="18"/>
+    <tableColumn id="1" xr3:uid="{26FE1E68-CD21-4445-80E0-A77866151FAB}" name="Khu vực" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{6D6F3738-0F8B-45BF-A515-A2A321F895EA}" name="Trạm" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{015C2645-BD78-45F2-98E9-00B03187980C}" name="Nguyên nhân" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{1175C761-AE1A-480A-9F1A-A8F410E010A6}" name="Hiện trạng / Đã xử lý" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C141E7F5-6026-4451-A09B-84C350D60D37}" name="b5_hung" displayName="b5_hung" ref="A3:D9" totalsRowShown="0" headerRowDxfId="17" headerRowBorderDxfId="16" tableBorderDxfId="15" totalsRowBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C141E7F5-6026-4451-A09B-84C350D60D37}" name="b5_hung" displayName="b5_hung" ref="A3:D9" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="5" tableBorderDxfId="6" totalsRowBorderDxfId="4">
   <autoFilter ref="A3:D9" xr:uid="{C141E7F5-6026-4451-A09B-84C350D60D37}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{727762F7-68BF-46A7-91B1-A3343CBBC224}" name="Khu vực" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{5F87AB82-8C4C-4ECF-B3A0-B064AB52CD12}" name="Trạm" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{9668A0CA-AC5F-4DAD-8A4C-79C8DBE5955C}" name="Nguyên nhân" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{2711B748-DF20-4E1A-9FE7-1428AB960E23}" name="Hiện trạng / Đã xử lý" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{727762F7-68BF-46A7-91B1-A3343CBBC224}" name="Khu vực" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{5F87AB82-8C4C-4ECF-B3A0-B064AB52CD12}" name="Trạm" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{9668A0CA-AC5F-4DAD-8A4C-79C8DBE5955C}" name="Nguyên nhân" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{2711B748-DF20-4E1A-9FE7-1428AB960E23}" name="Hiện trạng / Đã xử lý" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{06332DC4-D911-47DF-913E-C7A55424E9A7}" name="b6_hung" displayName="b6_hung" ref="A4:C10" totalsRowShown="0" tableBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{06332DC4-D911-47DF-913E-C7A55424E9A7}" name="b6_hung" displayName="b6_hung" ref="A4:C10" totalsRowShown="0" tableBorderDxfId="24">
   <autoFilter ref="A4:C10" xr:uid="{06332DC4-D911-47DF-913E-C7A55424E9A7}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{1C882C06-050F-476B-A538-6C6A411FAF9F}" name="STT" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{0E8485D0-8133-47FB-B4A4-6491F9317142}" name="Nội dung phản ánh / Tình trạng xử lý" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{E91BC7D4-881B-4D18-A14F-7AC890C85751}" name="Số lượng" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{1C882C06-050F-476B-A538-6C6A411FAF9F}" name="STT" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{0E8485D0-8133-47FB-B4A4-6491F9317142}" name="Nội dung phản ánh / Tình trạng xử lý" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{E91BC7D4-881B-4D18-A14F-7AC890C85751}" name="Số lượng" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{27EF9CBE-5A28-4C8C-B954-0C0C340C3712}" name="b7_hung" displayName="b7_hung" ref="A4:D8" totalsRowShown="0" headerRowDxfId="5" tableBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{27EF9CBE-5A28-4C8C-B954-0C0C340C3712}" name="b7_hung" displayName="b7_hung" ref="A4:D8" totalsRowShown="0" headerRowDxfId="13" tableBorderDxfId="12">
   <autoFilter ref="A4:D8" xr:uid="{27EF9CBE-5A28-4C8C-B954-0C0C340C3712}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{827B3220-FA6D-4A78-8E8C-38909574861D}" name="Khu vực" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{708DFEA4-B8DC-464B-8E36-C489ACCD6F7E}" name="Trạm" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{B1473778-DDD7-4AB1-847D-F909FE606643}" name="Nguyên nhân" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{BBB4DD37-9CC4-49B3-84C0-537CDF002998}" name="Hiện trạng / Đã xử lý" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{827B3220-FA6D-4A78-8E8C-38909574861D}" name="Khu vực" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{708DFEA4-B8DC-464B-8E36-C489ACCD6F7E}" name="Trạm" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{B1473778-DDD7-4AB1-847D-F909FE606643}" name="Nguyên nhân" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{BBB4DD37-9CC4-49B3-84C0-537CDF002998}" name="Hiện trạng / Đã xử lý" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3410,7 +3452,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BD7D8E2-4335-4199-A696-F8EAE90EA953}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" style="1" customWidth="1"/>
@@ -3425,7 +3467,7 @@
     <col min="10" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>117</v>
       </c>
@@ -3436,13 +3478,16 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-    </row>
-    <row r="2" spans="1:8" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2"/>
       <c r="B2"/>
       <c r="C2"/>
     </row>
-    <row r="3" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="37" t="s">
         <v>24</v>
       </c>
@@ -3468,7 +3513,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="18">
         <v>1</v>
       </c>
@@ -3494,7 +3539,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A5" s="13"/>
       <c r="B5" s="14"/>
       <c r="C5" s="22" t="s">
@@ -3508,7 +3553,7 @@
       <c r="G5" s="3"/>
       <c r="H5" s="14"/>
     </row>
-    <row r="6" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A6" s="13"/>
       <c r="B6" s="14"/>
       <c r="C6" s="22" t="s">
@@ -3522,7 +3567,7 @@
       <c r="G6" s="3"/>
       <c r="H6" s="14"/>
     </row>
-    <row r="7" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
       <c r="B7" s="14"/>
       <c r="C7" s="22" t="s">
@@ -3536,7 +3581,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="14"/>
     </row>
-    <row r="8" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
       <c r="B8" s="14"/>
       <c r="C8" s="22" t="s">
@@ -3550,7 +3595,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="14"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="16">
         <v>2</v>
       </c>
@@ -3576,7 +3621,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="13"/>
       <c r="B10" s="14"/>
       <c r="C10" s="22" t="s">
@@ -3590,7 +3635,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="14"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="B11" s="14"/>
       <c r="C11" s="22" t="s">
@@ -3604,7 +3649,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="14"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="59"/>
       <c r="B12" s="60"/>
       <c r="C12" s="61" t="s">
@@ -3629,7 +3674,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA11F483-9B58-4624-A05D-388937A5F6C7}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="1" customWidth="1"/>
@@ -3640,23 +3685,23 @@
     <col min="6" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1"/>
       <c r="B1"/>
       <c r="C1"/>
       <c r="D1"/>
     </row>
-    <row r="2" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2"/>
       <c r="B2"/>
       <c r="C2"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3"/>
       <c r="B3"/>
       <c r="C3"/>
     </row>
-    <row r="4" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="63" t="s">
         <v>0</v>
       </c>
@@ -3669,8 +3714,12 @@
       <c r="D4" s="65" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="63" x14ac:dyDescent="0.25">
+      <c r="E4" s="86" t="s">
+        <v>119</v>
+      </c>
+      <c r="F4" s="85"/>
+    </row>
+    <row r="5" spans="1:6" ht="63" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
         <v>4</v>
       </c>
@@ -3684,7 +3733,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A6" s="28" t="s">
         <v>8</v>
       </c>
@@ -3698,7 +3747,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A7" s="28" t="s">
         <v>12</v>
       </c>
@@ -3712,7 +3761,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A8" s="28" t="s">
         <v>15</v>
       </c>
@@ -3726,7 +3775,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>19</v>
       </c>
@@ -3738,7 +3787,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A10" s="66" t="s">
         <v>22</v>
       </c>
@@ -3751,6 +3800,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E4:F4"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -3760,7 +3812,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6FED11E-5217-4F35-B9B7-BBF6EF15C93F}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" customWidth="1"/>
@@ -3769,9 +3821,9 @@
     <col min="4" max="4" width="81.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:5" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="45" t="s">
         <v>0</v>
       </c>
@@ -3784,8 +3836,11 @@
       <c r="D3" s="47" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="63" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="63" x14ac:dyDescent="0.25">
       <c r="A4" s="69" t="s">
         <v>4</v>
       </c>
@@ -3799,7 +3854,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A5" s="69" t="s">
         <v>77</v>
       </c>
@@ -3813,7 +3868,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A6" s="69" t="s">
         <v>81</v>
       </c>
@@ -3827,7 +3882,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A7" s="69" t="s">
         <v>84</v>
       </c>
@@ -3841,7 +3896,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A8" s="69" t="s">
         <v>87</v>
       </c>
@@ -3855,7 +3910,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A9" s="71" t="s">
         <v>90</v>
       </c>
@@ -3986,7 +4041,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{143CF940-81A4-4373-AAC0-B9F739273311}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3995,20 +4050,20 @@
     <col min="4" max="4" width="70.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="79" t="s">
         <v>0</v>
       </c>
@@ -4021,8 +4076,12 @@
       <c r="D4" s="81" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="66" x14ac:dyDescent="0.25">
+      <c r="E4" s="88" t="s">
+        <v>120</v>
+      </c>
+      <c r="F4" s="87"/>
+    </row>
+    <row r="5" spans="1:6" ht="66" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>106</v>
       </c>
@@ -4036,7 +4095,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="33" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>22</v>
       </c>
@@ -4048,7 +4107,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="33" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>19</v>
       </c>
@@ -4060,7 +4119,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A8" s="82" t="s">
         <v>114</v>
       </c>
@@ -4075,6 +4134,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E4:F4"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>